<commit_message>
update text generation files
</commit_message>
<xml_diff>
--- a/src/data_collection/sv_data_collection.xlsx
+++ b/src/data_collection/sv_data_collection.xlsx
@@ -5,16 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lawcs-my.sharepoint.com/personal/gwelsh_tullius_com_au/Documents/Thesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lawcs-my.sharepoint.com/personal/gwelsh_tullius_com_au/Documents/Thesis/CLUU-thesis/src/data_collection/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="400" documentId="8_{2F4FE38B-AA2A-4D5D-9029-C89C327E4BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D13B07CB-A67A-4020-80A0-C1735AB0F9E4}"/>
+  <xr:revisionPtr revIDLastSave="401" documentId="8_{2F4FE38B-AA2A-4D5D-9029-C89C327E4BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FEB8DE4-9345-4801-B2E6-BEBC40226524}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{48665015-FE5C-4201-9A77-615E45CC6C6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Abstracts" sheetId="1" r:id="rId1"/>
-    <sheet name="Reddit_Comments" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Abstracts!$A$1:$G$1</definedName>
@@ -2163,13 +2162,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId12"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0803377F-952C-43BD-8CEE-CFA48D594A6B}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
update llm generated abstracts
</commit_message>
<xml_diff>
--- a/src/data_collection/sv_data_collection.xlsx
+++ b/src/data_collection/sv_data_collection.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lawcs-my.sharepoint.com/personal/gwelsh_tullius_com_au/Documents/Thesis/CLUU-thesis/src/data_collection/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="401" documentId="8_{2F4FE38B-AA2A-4D5D-9029-C89C327E4BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FEB8DE4-9345-4801-B2E6-BEBC40226524}"/>
+  <xr:revisionPtr revIDLastSave="411" documentId="8_{2F4FE38B-AA2A-4D5D-9029-C89C327E4BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{860A940E-C5DD-412D-BD6F-EEA870FDEE3B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{48665015-FE5C-4201-9A77-615E45CC6C6B}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{48665015-FE5C-4201-9A77-615E45CC6C6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Abstracts" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Abstracts!$A$1:$G$1</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="261">
   <si>
     <t>Level</t>
   </si>
@@ -724,12 +725,324 @@
   <si>
     <t>https://www.diva-portal.org/smash/get/diva2:712460/FULLTEXT01.pdf</t>
   </si>
+  <si>
+    <t>Generated Abstract</t>
+  </si>
+  <si>
+    <t>Målet med studien är att bidra med vägledning kring vilka gröna nyckeltal som kan vara relevanta och användbara för mindre företags redovisning. Vi undersöker om drivkrafterna bakom miljörapportering kan identifieras och på vilket sätt intressenter påverkar utvecklingen. För att fånga tendenser inom området används även större företagsgrupper som jämförelse för att illustrera olika angreppssätt och ge exempel på miljöarbete. Den teoretiska delen beskriver först möjliga motiv till miljöredovisning och fördjupar sig därefter i begreppet gröna nyckeltal. Vidare presenteras intressentperspektivet och legitimitetsteorin samt hur olika intressenter nyttjar miljöinformation.</t>
+  </si>
+  <si>
+    <t>Generated_Abstract</t>
+  </si>
+  <si>
+    <t>Målet med denna uppsats är att undersöka på vilka sätt föreställningen om ett narkotikafritt samhälle tar form i diskurser där narkotikamissbruk beskrivs som ett socialt problem. Som empiriskt underlag används ett policydokument och en debattserie, vilka analyseras med utgångspunkt i socialkonstruktivism och diskursanalys. Resultaten indikerar att en pågående definitionskamp om hur narkotikamissbruk ska förstås sträcker sig över flera diskurser, där visionen om det narkotikafria samhället samtidigt återkommer som en central referenspunkt. En nationell diskurs framträder, kopplad till föreställningar om vad “vi” som land vill och bör vara. En moraldiskurs som värderar handlingar, livsstilar och ställningstaganden. Därtill syns en juridisk och polisiär diskurs som, med narkotikans rättsliga status som utgångspunkt, avgränsar och strukturerar problemet, samt en barn- och ungdomsdiskurs som positionerar narkotika som ett överordnat hot. Sammantaget visar studien hur dessa diskurser samverkar i konstruktionen av narkotikamissbruk som socialt problem.</t>
+  </si>
+  <si>
+    <t>Arbetslivets utveckling med ökat tempo, fler tidsbegränsade anställningar och större krav på flexibilitet gör att en växande andel arbetstagare upplever stress. Vid långvarig belastning ökar risken för ohälsa hos individen. Då en stor del av dagens sjukskrivningar kopplas till stressrelaterade tillstånd, exempelvis depression och utmattningssyndrom, är det angeläget att undersöka verksamma strategier för stresshantering på arbetsplatsen. Beröring, såsom massage, har visats kunna dämpa stress och kan även fungera som ett komplement vid behandling av stressrelaterade besvär. I ett fältexperiment med 28 tjänstemän prövades om en kort massage under arbetstid kunde minska arbetsrelaterad stress jämfört med en avslappningsövning och en ordinarie rast. Resultaten visade en signifikant sänkning av stressnivåerna efter massageinsatsen. Sammantaget tyder fynden på att upplevd stress kan reduceras genom fysisk beröring. Studien diskuterar även urvalets storlek samt möjliga förväntanseffekter som kan ha påverkat resultaten.</t>
+  </si>
+  <si>
+    <t>Syftet med denna studie är att skapa en fördjupad förståelse för hur pedagoger uppfattar och vidareutvecklar arbetet med begreppet hållbar utveckling utifrån sin befintliga kunskap. Som teoretisk utgångspunkt används perspektiv på kunskap och hållbar utveckling samt begreppet handlingskompetens. Studien genomförs med en kvalitativ ansats och bygger på semistrukturerade intervjuer med totalt sex pedagoger verksamma vid två förskolor i södra Sverige. Arbetet tar sin utgångspunkt i två forskningsfrågor: (1) hur relaterar pedagoger till hållbar utveckling ur ett lärandeperspektiv, samt (2) i de fall normer och värderingar blir synliga, på vilka sätt kommer dessa till uttryck i pedagogernas arbete med kunskapsbildning för hållbar utveckling. Resultaten visar att pedagogernas förståelse av hållbar utveckling främst kopplas till de tre dimensionerna ekologisk, ekonomisk och social. Kunskapsbildningen tycks i stor utsträckning ha sin grund i fortbildningsinsatsen Grön flagg eller i pedagogernas personliga engagemang. Lärandet för hållbar utveckling sker framför allt genom områden som kan göras konkreta och vardagsnära för barnen, exempelvis sortering av avfall och skräpplockning. Pedagogerna beskriver även situationer där barns handlingskompetens framträder. De framhåller sin roll som förebilder i arbetet. I beskrivningarna dominerar en normerande undervisningsform, där attityder och värderingar påverkar och styr om och hur handlingar för hållbar utveckling genomförs.</t>
+  </si>
+  <si>
+    <t>I den här studien har jag undersökt handledning i arbetslivet. Handledning är i dag ett relativt svårfångat begrepp som samtidigt får en allt tydligare plats på många arbetsplatser. Arbetets syfte är att belysa vad handledning kan innebära, hur olika handledningsprocesser ser ut och på vilka sätt dessa skulle kunna tillämpas i organisationer, särskilt i samband med medarbetarsamtal. Jag avgränsar undersökningen till den del av medarbetarsamtalet som handlar om individens utveckling. Min teoretiska utgångspunkt är att handledande inslag kan förekomma i medarbetarsamtalet, men att hela samtalet inte utan vidare kan beskrivas som handledning. För att studera detta har jag genomfört intervjuer med åtta personer på två arbetsplatser; fyra chefer och fyra medarbetare, där fokus har varit erfarenheter av medarbetarsamtalet. Resultaten visar att ett handledande förhållningssätt tydligt går att identifiera i samtalen på båda arbetsplatserna, och att metoder och perspektiv från handledningsfältet kan bidra till att vidareutveckla medarbetarsamtalet. Om medarbetarsamtalet inte betraktas som handledning i sin helhet, men som en situation där handledning kan initieras, kan det snarare förstås som en utgångspunkt för den fortlöpande handledning som sker i det dagliga arbetet. Samtalet blir då ett tillfälle att klargöra förväntningar, enas om utvecklingsbehov och få en gemensam bild av arbetssituationen, vilket sedan kan följas upp och omsättas i praktiken fram till nästa medarbetarsamtal.</t>
+  </si>
+  <si>
+    <t>I *Samkönade äktenskaps vara eller icke vara inom Svenska kyrkan* genomförs en argumentationsanalys, med hermeneutisk ansats och kvalitativ textanalys, av debattinlägg om huruvida Svenska kyrkan bör behålla vigselrätten efter att staten gjort äktenskapslagstiftningen könsneutral. Materialet består av artiklar publicerade 2008-12-11 till 2009-10-31 i *Kyrkans tidning* och *Dagens Nyheter*. Resultatet visar att både förespråkare och motståndare i stor utsträckning använder likartade argumenttyper, men ger dem skilda innebörder genom olika betoningar och tolkningar. Motståndarsidan lutar dock oftare mot ett toleransresonemang än ja-sidan. I ja-sidans argumentation framträder samtidigt en implicit normkritik riktad mot heteronormativiteten.</t>
+  </si>
+  <si>
+    <t>I studien relateras läroplanernas krav på undervisning som berör intersektionalitet till det innehåll som återfinns i religionskunskapsläroböcker för gymnasiet utgivna efter gymnasiereformen 2011. Syftet var att undersöka om läroböckerna behandlar intersektionalitet explicit eller mer underförstått, och/eller om kategorierna kön, sexualitet, socioekonomiska villkor och etnicitet främst framställs var för sig, samt i vilka sammanhang detta i så fall sker. Tre forskningsfrågor utformades. Den första rörde hur religionsläroböcker publicerade från 2011 och framåt beskriver relationen mellan världsreligionerna och kategorierna kön, sexualitet, socioekonomisk bakgrund och etnicitet. Den andra frågan avsåg i vilka andra delar av böckerna (exempelvis kapitel) dessa kategorier behandlas. Den tredje frågan fokuserade på vad läroböckerna tar upp om begreppet och fenomenet intersektionalitet.</t>
+  </si>
+  <si>
+    <t>Denna uppsats undersöker Paulus förståelse av lagen, ett av de mest omstridda fälten inom paulusforskningen. Frågan om hur Paulus förhåller sig till lagen är så avgörande för helhetstolkningen av hans teologi att den som vill tolka Paulus och hans brev behöver ta ställning i ämnet. Litteraturen är omfattande och debatten tycks fortfarande vara långt ifrån avgjord. Samtidigt kräver en sådan problematik tydliga avgränsningar för att kunna hanteras inom ramen för en kortare studie. Därför avgränsas undersökningen till en specifik perikop i ett av Paulus brev där temat står i centrum. Uppsatsens huvudfråga formuleras så: Vad avser Paulus med uttrycket ”lagen” i Rom 3:21–31?</t>
+  </si>
+  <si>
+    <t>Denna studie behandlar teologiska tolkningar av två kungar som tillskrevs gudomlig status i det forntida Mesopotamien: den gammalakkadiske Naram-Sin (ca 2254–2218 f.Kr.) och den nysumeriske Shulgi (ca 2094–2047 f.Kr.). Perspektiven analyseras genom en induktivt orienterad historisk genomgång som tar sin utgångspunkt i tidigare forskning om ämnet. Eftersom arbetet är en c-uppsats och tillgången till primärmaterial (såsom arkeologiska fynd och källtexter på originalspråk) har varit begränsad, baseras undersökningen helt på sekundärlitteratur. Framställningen är uppdelad i tre avsnitt: två där respektive kung behandlas separat utifrån forskningsläget, och ett tredje där resultaten ställs mot varandra i en jämförande analys. Metoden har varit att först sammanställa vad forskare faktiskt hävdar om de teologiska föreställningarna kring monarkerna, därefter dela upp materialet i återkommande delteman och sortera utsagorna efter dessa. På grundval av detta försöker studien teckna en övergripande bild av perspektivens karaktär och deras huvudsakliga inriktningar. Tyngdpunkten ligger på att identifiera mönster i de religiösa idéerna och vilka motiv de främst kretsar kring. Resultatet visar att tolkningarna är mångfacetterade och delvis motstridiga, men att både skillnader och överlappningar kan urskiljas mellan kungarna. Två motiv som återkommer särskilt ofta är fruktbarhet och föreställningar kopplade till himlen.</t>
+  </si>
+  <si>
+    <t>Denna studie undersöker hur lärarstudenter och yrkesverksamma lärare ställer sig till skolavslutningar och högtidsfiranden i kyrkan, samt till motsvarande arrangemang när de innehåller konfessionella moment. Empirin bygger på en webbaserad enkät som besvarats av både blivande och aktiva lärare. Resultaten visar att en majoritet i båda grupperna är positivt inställda till att använda kyrkorummet som plats för dessa aktiviteter. Samtidigt är den största andelen negativa till att inslagen har en konfessionell karaktär. Äldre deltagare uppvisar generellt en mer positiv hållning, både till kyrkomiljön och till religiösa inslag, jämfört med yngre. Sammantaget pekar slutsatserna mot en fortsatt sekulariseringsutveckling i Sverige i enlighet med reviderade sekulariseringsteorier, eftersom konfessionalitet i regel inte efterfrågas av flertalet lärare och lärarstudenter. Det framträder dock även tydliga undantag från detta mönster. Kyrkan tycks samtidigt behålla en i huvudsak sekulär och traditionsburen funktion inom skolans sammanhang, vilket gör den fortsatt betydelsefull.</t>
+  </si>
+  <si>
+    <t>En betydande del av Sveriges bostadsbestånd uppfördes under åren 1965–1974 som en följd av den akuta bostadsbristen. För att möta behovet fattade staten beslut om att bygga en miljon bostäder under perioden, det som kom att kallas miljonprogrammet. Byggandet omfattade olika typer av bostäder i skilda storlekar, men områdena präglas ofta av storskalighet och återkommande, likartade hus. I dag står många av dessa byggnader inför omfattande renoveringsbehov. Eftersom bebyggelsen ses som kulturhistoriskt intressant och representativ för en period i svensk arkitektur, ställer kommuner särskilda krav när åtgärder planeras. Det kommunala bostadsbolaget Gavlegårdarna i Gävle har därför tagit initiativ till att utveckla bygglovsprocessen för renoveringar i sådana områden. Syftet är att korta tiden fram till ett beviljat bygglov och att göra dialogen med kommunen mer effektiv genom hela projektet. För att i största möjliga utsträckning bevara områdets karaktär har Gavlegårdarna tagit fram en arbetsmodell där en extern bevarandespecialist anlitas som länk mellan bolaget och kommunen, samt som stöd med erfarenheter kopplade till platsens värden. Därtill involveras kommunen tidigt, redan vid den första presentationen av förslaget, vilket gör att synpunkter kan integreras innan bygglovsansökan lämnas in.</t>
+  </si>
+  <si>
+    <t>Rapporten är en reflekterande genomgång av mitt och Petri Tuoris gemensamma examensarbete London Crysis, framtaget vid Högskolan i Skövde. Projektet är byggt i spelet Crysis och skildrar en fiktiv version av London under 1800-talet, med tydliga influenser från bland annat From Hell och Sweeney Todd: The Demon Barber of Fleet Street. Texten inleds med en bakgrund som redogör för verkets ursprung, dess problemformulering, syfte samt vilka avgränsningar som gjorts. Därefter följer en presentation av produktionen med fördjupning kring idéutveckling, leveldesign, atmosfär, exempel på modeller samt arbetet med webbplats och trailer. Rapporten beskriver även den enkätundersökning som genomfördes för att undersöka hur andra uppfattar spelets stämning och vilka tolkningar som uppstår. Avslutningsvis förs en sammanfattande diskussion där enkätens resultat vägs mot målen med verket och de erfarenheter projektet gav.</t>
+  </si>
+  <si>
+    <t>Detta arbete utforskar hur svenskt teckenspråk, återgivet virtuellt, upplevs av teckenspråksanvändare i en datorspelskontext. I en empirisk studie prövades flera sätt att presentera teckenspråk i tredjepersonsvy. Bakgrunden tar upp aktuella tillämpningar av virtuellt teckenspråk och avatarer samt frågor om inkludering, animation, spelkameror och svenskt teckenspråk. Studien syftar till att besvara vilket perspektiv som svenska teckenspråksanvändare föredrar när teckenspråk integreras i spel. Artefakten bestod av tre videobaserade spelsimuleringar med 3D-animerade sekvenser, som deltagarna fick rangordna utifrån teckenspråkets tydlighet och utifrån vilket perspektiv de helst skulle vilja se i ett teckenspråksanpassat spel. Deltagarurvalet utgjordes av svenska teckenspråksanvändare; totalt besvarade 51 personer en enkät. Av dessa uppgav 27 en funktionsvariation, 16 hade en närstående med funktionsvariation och resterande deltog utifrån intresse. Resultaten kan ligga till grund för vidare forskning som utvecklar mer inkluderande speldesign och ökar tillgängligheten för teckenspråksanvändare.</t>
+  </si>
+  <si>
+    <t>Under de senaste åren har 3D-visualisering blivit ett allt vanligare verktyg i kommunal fysisk planering. I kombination med att jag själv arbetar med tekniken i min roll som planarkitekt väcktes frågor om varför den införts, vilka beslut och förväntningar som drivit utvecklingen samt vilket vetenskapligt stöd som finns för att 3D bidrar till bättre visualisering, tydlighet och kommunikation i planprocessen. Detta examensarbete i Fysisk planering vid BTH syftar till att undersöka dessa aspekter. Studien bygger på en litteraturgenomgång av relevant forskning, en enkät till ett mindre urval tjänstepersoner och politiker i fyra kommuner som ingår i ett 3D-nätverk, en genomgång av samma kommuners webbdokumentation samt en kompletterande enkät riktad till planarkitekter i fem andra kommuner som står utanför nätverket. Det konstateras att det saknas tydligt forskningsstöd som visar på effektivitet, eller som systematiskt väger för- och nackdelar, med 3D-modeller för ökad förståelse och förbättrad kommunikation mellan tjänstepersoner, politiker och allmänhet i kommunal planering. Genom att sammanföra resultat från miljöpsykologi, planredovisning/visualisering och svensk arkitekturforskning framträder ändå indikationer på både möjligheter och begränsningar i 3D-visualiseringens roll som kommunikationsmedel. Använd på ett genomtänkt sätt kan tekniken stärka åskådliggörandet, men den medför samtidigt risker kopplade till hur och när visualiseringar används. Som främsta motiv till införande anges – av planarkitekter, ansvariga tjänstepersoner och politiker – en ambition att öka medborgarnas förståelse för förändringsförslag i den byggda miljön, vilket i de fall dokument finns också ofta speglas i kommunernas formuleringar. Samtidigt saknar flera kommuner fastställda riktlinjer och policydokument på området. Forskningen pekar dessutom på särskilda risker med visualisering i planprocessens tidiga skeden. I den avslutande diskussionen behandlas studiens frågeställningar, möjliga problem och potentialer med 3D-tekniken samt förslag på fortsatt forskning. Slutsatsen är att en tydlig skillnad finns mellan kommunernas överlag positiva bild av nyttan och de mer problematiserande resultat som framkommer i forskningen.</t>
+  </si>
+  <si>
+    <t>I den snabbt expanderande e-handeln är konkurrensen hård, och behovet av att hitta nya sätt att öka försäljningen och stärka marknadspositionen är stort. Denna studie undersöker användningen av stereoskopisk 3D som metod för produktpresentation. En tydlig fördel är att tekniken kan ge konsumenten en mer realistisk uppfattning av varan än traditionella tvådimensionella produktbilder. Den mest framträdande förbättringen gäller djupkänslan, vilket tycks underlätta bedömningen av en produkts volym och rymd. Samtidigt är stereoskopisk 3D i princip outnyttjad inom e-handel, vilket motiverar en analys av möjliga orsaker. En sannolik förklaring är att tekniken fortfarande är relativt ny och därför inte fullt mogen. Resultaten visar exempelvis att deltagare ofta uppfattar 2D-bilder som skarpare än 3D-bilder. Flera andra visuella egenskaper som bedömts utifrån bilder fick också lägre omdömen i 3D-gruppen jämfört med 2D-gruppen. Däremot uppvisar egenskaper som hänger samman med djupupplevelse en tydligt positiv koppling till 3D-visning. Studien pekar även på att upplevelsen av 3D påverkas av hur utvärderingen genomförs. I ett tänka-högt-test uttryckte deltagarna en mer positiv inställning till 3D-bilder än vad som framkom i en mer omfattande enkät i ett efterföljande test.</t>
+  </si>
+  <si>
+    <t>I början av 1980-talet började man rapportera om sällsynta tumörer och opportunistiska infektioner hos unga män, tillstånd som annars främst ses hos personer med kraftigt nedsatt immunförsvar. År 1983 och 1984 identifierade forskarteam i Frankrike respektive USA ett tidigare okänt virus, som senare fick beteckningen humant immunbristvirus (HIV). HIV-infektion kan fortgå i många år utan tydliga symtom, och först när immunförsvaret successivt försvagas blir sjukdomstecken märkbara. Det första läkemedlet mot HIV godkändes 1987, vilket bidrog till en tydlig minskning av dödligheten i det AIDS-relaterade sjukdomsförloppet. År 1996 introducerades därefter en behandlingsprincip med kombinationer av tre eller fler preparat, som blev känd som antiretroviral terapi (ART).</t>
+  </si>
+  <si>
+    <t>Förekomsten av allergiska sjukdomar har ökat markant sedan mitten av 1900-talet. Allergenspecifik immunterapi är en immunmodulerande behandlingsform som kan övervägas vid medelsvår till svår IgE-medierad allergi och ges antingen sublingualt eller subkutant. Detta litteraturarbete syftade till att klarlägga om sublingual immunterapi (SLIT) och subkutan immunterapi (SCIT) med husdammskvalsterallergen skiljer sig åt avseende förändringar i symtom- och medicineringspoäng samt nivåer av specifika IgE- och IgG4-antikroppar, IL‑10 och IFN‑γ. Litteratursökning genomfördes i PubMed. Fem studier som utvärderade effekten av både SLIT och SCIT inkluderades. I studie 1 och 2 sågs en signifikant större minskning av astmasymtom med SCIT, medan motsvarande skillnad inte kunde påvisas i studie 3. Astmans medicineringspoäng minskade i högre grad med SCIT än SLIT i studie 2, men inte i studie 1. I studie 4 minskade symtompoängen signifikant mer med SCIT jämfört med SLIT. För rinit sågs ingen statistiskt säkerställd skillnad mellan behandlingsformerna avseende symtompoäng i studie 1–3, medicineringspoäng i studie 1 och 2 eller total medicineringspoäng i studie 3. SCIT gav en signifikant större ökning av specifikt IgG4 än SLIT i studie 1, 2 och 5. Däremot framkom ingen signifikant skillnad mellan SLIT och SCIT avseende förändringar i specifikt IgE, IL‑10 eller IFN‑γ. Sammantaget indikerar resultaten att SLIT och SCIT ger likvärdig förbättring av rinit vad gäller symtom och läkemedelsbehov efter 1–2 års behandling, medan SCIT möjligen ger bättre effekt efter 3 år. För astma förefaller SCIT överlag vara mer effektiv än SLIT. SCIT tycks dessutom inducera en kraftigare IgG4-respons. Ytterligare randomiserade kontrollerade studier med direkt jämförelse mellan SLIT och SCIT behövs för att avgöra om eventuella skillnader i långtidseffekt vid husdammskvalsterimmunterapi är bestående.</t>
+  </si>
+  <si>
+    <t>I Sverige är abort tillåtet och flera metoder för regelbunden preventivmedelsanvändning är etablerade, men trots detta kvarstår behovet av akut prevention vid risk för oplanerad graviditet. Det finns tre godkända alternativ för akutpreventivmedel: levonorgestrel, ulipristalacetat och kopparspiral. Syftet med detta arbete var att sammanställa och bedöma effektivitet och säkerhet för dessa tre metoder. En litteratursökning genomfördes i PubMed och totalt inkluderades sju artiklar för analys. I artikel 1 och 2 studerades levonorgestrel, där graviditetsfrekvensen rapporterades till 0,57 % respektive 0,67 %, samt en uppskattad graviditetsförebyggande effekt på 68 %. Artikel 3 jämförde ulipristal med levonorgestrel och visade graviditetsfrekvenser på 1,8 % för ulipristal och 2,6 % för levonorgestrel, med stöd för non-inferiority (OR 0,68). Artikel 4 utvärderade levonorgestrel vid olika tidpunkter och redovisade graviditetsfrekvens 2,0 % i 12-timmarsgruppen och 1,9 % i 24-timmarsgruppen, samt effekt på 72 % respektive 75 %. Artikel 5 fann vid jämförelse att ulipristal var non-inferior till levonorgestrel. Artikel 6 rapporterade för ulipristal en graviditetsfrekvens på 2,1 % och en graviditetsförebyggande effekt på 62,3 %. Artikel 7 analyserade kopparspiral och redovisade 100 % graviditetsförebyggande effektivitet. Sammanfattningsvis är akutpreventivmedel inte helt tillförlitliga, men minskar risken för oönskad graviditet avsevärt. Resultaten bedöms vara förenliga med nuvarande behandlingsrekommendationer.</t>
+  </si>
+  <si>
+    <t>Globala mattrender påverkar bageribranschen och användningen av fröer i livsmedel har ökat markant under senare år. Trots detta utnyttjas fortfarande ett relativt litet urval fröer i dagens brödproduktion, och det finns därför intresse för att identifiera nya alternativ som kan tillföra både funktion och mervärde. Detta examensarbete syftar till att undersöka amarant, bovete, chia, hirs och quinoa, med fokus på vilka näringsmässiga och sensoriska egenskaper de kan bidra med i bröd. Arbetet genomförs i samarbete med Pågen AB. Med stöd av en mindre litteraturgenomgång och praktiska bakförsök, följt av analyser av brödvolym, inkråm, textur och vattenhalt, utvärderas fröernas bakegenskaper och potentiella användningsområden. Sensoriska bedömningar genomförs också för att kartlägga smak, doft och helhetsintryck för respektive frö. Utifrån resultaten valdes chia, bovete och quinoa ut för fortsatta försök. Chia och bovete prioriterades bland annat tack vare positiva sensoriska utfall, och testerna indikerade att båda kan användas i flera brödtyper och i varierande dosering. Quinoa uppvisade en påtaglig bitterhet i smak och arom som var svår att eliminera, men som minskade när fröet användes som topping. Även chia och krossat bovete fungerade väl som dekor på bröd. Sammantaget visar studien att det finns lovande alternativa fröer som kan bidra till både näringsprofil och smakupplevelse. För att bedöma deras lämplighet i storskalig produktion behövs dock fler försök med olika recept och frömängder.</t>
+  </si>
+  <si>
+    <t>Sepsis är ett potentiellt livshotande tillstånd som kan uppstå när bakterier sprids från en lokal infektion till blodbanan. Vid positiva blododlingar odlas mikroorganismer på agar, varefter identifiering kan göras med Matrix Assisted Laser Desorption Ionisation Time-of-Flight Mass Spectrometry (MALDI‑TOF MS). I metoden blandas provet med en matrix och bestrålas med laser så att proteiner joniseras och accelereras mot en detektor. Resultatet blir ett masspektrum (m/z) som jämförs mot referensprofiler i en databas, och ett score anger hur väl provet överensstämmer med referensen. Syftet med arbetet var att utvärdera om bakterier kan direktidentifieras från blod efter en specifik provberedning inför MALDI‑TOF MS för att möjliggöra snabbare preliminära svar, samt att bedöma om metoden kan skilja Staphylococcus aureus från koagulasnegativa stafylokocker. Inför analys preparerades blod från positiva blododlingar genom stegvis centrifugering med 5 % natriumkloridlösning (NaCl‑metoden). Därutöver prövades ett kommersiellt prepareringskit (Sepsityper, Bruker Daltonics). Med NaCl‑metoden uppnåddes korrekt artidentifiering i 66 % av de inokulerade proverna. För blododlingar med S. aureus respektive koagulasnegativa stafylokocker identifierades 60 % respektive 43 % korrekt. Med Sepsityper erhöll 58 % av proverna ett godkänt score. Sammantaget visar resultaten att direktidentifiering från blod är möjlig efter provberedning, men att metoden behöver vidareutvecklas eftersom signifikanta skillnader i score sågs jämfört med nuvarande rutin. Däremot verkar det vara genomförbart att särskilja S. aureus från koagulasnegativa stafylokocker. Ytterligare studier krävs för att bedöma om någon av metoderna kan införas i rutindiagnostik.</t>
+  </si>
+  <si>
+    <t>Under förskoleåldern behöver barn bygga upp en förståelse för tal, samtidigt som de tillägnar sig det talade språket. Barns förutsättningar att utveckla matematiska kunskaper påverkas av hur de tidigt möter matematiken i vardag och undervisning. Denna uppsats är en fallstudie med syftet att beskriva hur The English School i Älmhult arbetar med att stärka barns taluppfattning. För att skapa en så nyanserad bild som möjligt har vi genomfört observationer samt intervjuat de två lärare som arbetar med åldersgruppen och även skolans rektor. Därutöver har vi granskat de styrdokument som, vid sidan av Lpfö 98, utgör grund för verksamheten. Studien visar en miljö där matematiken synliggörs och prioriteras redan tidigt. Lärarna arbetar medvetet och systematiskt med att presentera och introducera matematiska begrepp för barnen.</t>
+  </si>
+  <si>
+    <t>Detta arbete analyserar hur två olika nätverksarkitekturer för artificiella neurala nätverk presterar i en testmiljö med shooter-liknande karaktär. De arkitekturer som jämförs är ett traditionellt feedforward-nätverk och ett Elman-nätverk, där båda tränas med evolutionära algoritmer. Den centrala skillnaden mellan dem är att Elman-nätverket är rekurrent och därmed kan utnyttja ett korttidsminne.</t>
+  </si>
+  <si>
+    <t>Resultaten indikerar att det i den använda testmiljön inte framträder någon tydlig prestandaskillnad mellan arkitekturerna</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> då de i stort sett når likvärdiga resultat. Samtidigt visar de beteenden som agenterna utvecklar att neurala nätverksbaserade agenter kan fungera väl i ett shooter-spel och åstadkomma goda prestationer. Frågor som inte behandlats här men som vore relevanta för framtida studier är exempelvis hur nätverkens storlek påverkar utfallet</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> eller om ett rekurrent nätverk med mer långsiktig minnesförmåga skulle kunna ge andra resultat."</t>
+  </si>
+  <si>
+    <t>I takt med att datorspel blir allt mer visuellt avancerade ökar också behovet av lagringsutrymme för att rymma stora mängder bildtexturer. Detta kan göra att titlar som annars hade kunnat distribueras via exempelvis XBOX Live Marketplace blir för omfattande för plattformens storleksbegränsningar. Ett sätt att minska denna datamängd är att ersätta traditionella, lagrade texturer med procedurellt genererade texturer, vilka i regel kräver betydligt mindre utrymme. I denna uppsats presenteras och utvärderas en metod för att rekonstruera bildtexturer som procedurella varianter, där en genetisk algoritm används för att successivt evolvera fram texturer som visuellt liknar en given referenstextur.</t>
+  </si>
+  <si>
+    <t>Studien i denna rapport undersöker ansiktsigenkänning i realtid med webbkamerabilder genom att kombinera principal component analysis (PCA) med feedforward-baserade artificiella neurala nätverk. Metoden vidareutvecklas genom att integrera filterbaserade angreppssätt, inspirerade av tekniker inom ansiktsdetektering. Filtren utnyttjar redundans genom att även inkludera information från flera delområden i ansiktet för att stärka igenkänningens robusthet.</t>
+  </si>
+  <si>
+    <t>Sverige har under senare år ställts inför ett växande mottagande av ensamkommande barn. I sådana situationer blir det centralt att myndigheter och kommuner kan fatta likvärdiga beslut med stöd av ändamålsenliga beslutsstödsystem. Denna studie granskar arbetssätt hos Migrationsverket och två kommuner utifrån frågan: ”Hur används beslutsstödsystem vid placering av ensamkommande barn i kommuner?”. Ansatsen är kvalitativ, där empiri har samlats in genom litteraturstudier och intervjuer. Under studiens olika faser har Zachmans ramverk använts för att strukturera analysen av materialet samt som stöd vid utformning av intervjufrågor och genomförande av intervjuer. Respondenternas utsagor har därefter analyserats med hjälp av en beslutsmodell och Zachmans ramverk för att tydliggöra hur processer och roller förhåller sig till dessa modeller. Resultaten visar ett uttalat behov av ökad effektivitet i kommunernas beslutsfattande och i hur information från Migrationsverket tas emot. Kommunerna beskriver i nuläget sina beslutsprocesser som i hög grad manuella. Ur ett Business Intelligence (BI)-perspektiv drar studien slutsatsen att Migrationsverket och kommunerna behöver utveckla ett mer dynamiskt samspel kring beslutsfattande, integration samt informationsdelning och informationshantering för att möjliggöra bättre beslut. Studien kan fungera som utgångspunkt för vidare forskning om hur BI-behov kan identifieras och implementeras i verksamheter genom tillämpning av Zachmans ramverk.</t>
+  </si>
+  <si>
+    <t>Matsvinnet i Sverige beräknas uppgå till omkring en miljon ton årligen, och mycket tyder på att den största andelen uppstår i hushållen. Nya data pekar på att upp till cirka 100 kilo mat per person och år kastas, vilket medför betydande och i stor utsträckning onödiga konsekvenser för klimat och miljö. Att minska matsvinnet kan därför bidra till att reducera denna belastning. Denna studie har haft som mål att undersöka svenska hushålls inställningar till matsvinn samt att tydliggöra vilka hinder och möjligheter som påverkar förutsättningarna för att minska svinnet. Studien baseras på sju individuella konsumentintervjuer. Resultaten indikerar att deltagarna inte tycker om att kasta mat och uppger att de slänger förhållandevis små mängder. Miljöargument framstår dock inte som den viktigaste drivkraften bakom deras vilja att undvika svinn. Snarare lyfts värderingar som att visa omtanke om maten, solidaritet med mindre bemedlade och hänsyn till den egna ekonomin. Dessa perspektiv verkar ha grundlagts under uppväxten och, tillsammans med praktiska färdigheter i matlagning, utgöra centrala faktorer som hänger samman med lägre matsvinn.</t>
+  </si>
+  <si>
+    <t>Bakgrund Den gravida kvinnans kost är central eftersom näringsbehovet ökar och hon samtidigt påverkar fostrets utveckling. Grunden för barnets kommande hälsa och matpreferenser kan delvis etableras redan under fosterlivet. Samtidigt visar tidigare forskning att många gravida inte når upp till kostrekommendationerna och att konsumtionen av sötsaker och fikaprodukter ofta stiger. Studiens syfte var att undersöka hur nyblivna förstagångsmammor såg på hälsosamma respektive ohälsosamma livsmedel under graviditeten, samt hur dessa uppfattningar upplevdes påverka deras faktiska ätande. Åtta nyblivna förstagångsmammor intervjuades. Intervjuerna genomfördes med semistrukturerade frågor, spelades in via en inspelningsapplikation, transkriberades ordagrant och analyserades med kvalitativ innehållsanalys. Deltagarna beskrev att graviditeten ledde till en förändrad syn på mat. Det upplevdes viktigare att äta mer varierat med större inslag av frukt och grönsaker (hälsosam mat), medan intaget av snabbmat och sockerhaltiga produkter minskade (ohälsosam mat). Denna förändring var dock inte stabil över tid; senare i graviditeten rapporterades en ökning av snabbmat och söta livsmedel. Råd från vårdpersonal uppfattades som otillräckliga, både genom att informationen var begränsad och genom att deltagarna själva behövde söka kunskap, framför allt via Livsmedelsverket. Sammantaget framkom att den initiala ambitionen kring hälsosam respektive ohälsosam mat inte upprätthölls genom hela graviditeten, och att deltagarna önskade mer konkret vägledning från vården. Utökat stöd och tydligare kostinformation kan stärka den gravida kvinnans möjligheter att bibehålla hälsosamma matvanor under hela graviditeten.</t>
+  </si>
+  <si>
+    <t>Forskning har visat att hur länge barn ammats, har betydelse för deras hälsa senare i livet. Även barnens sociala miljö har visat sig ha effekt på hälsan och barnens matvanor. Salut är en satsning av Västerbottens läns landsting med målet att förbättra länsbornas hälsa fram till 2030. Syftet med studien var att undersöka treåringars matvanor, Body Mass Index (BMI) och fysiska aktivitet i relation till amningsduration och familjekonstellation.</t>
+  </si>
+  <si>
+    <t>Studien genomfördes genom ett samarbete med Salut som utformade och delade ut en enkät via barnavårdscentraler till samtliga föräldrar vid treårskontrollen. Enkäten innehöll frågor om barnens fysiska och psykiska hälsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> samt livsstil och levnadsvanor och totalt beabetades 210 av enkäterna i denna studie</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> där 16 frågor valdes ut. Dessa analyserades sedan statistiskt i IBM SPSS 21.0 Statistics. Signifikansnivån sattes till p&lt;0</t>
+  </si>
+  <si>
+    <t>05. De flesta av barnen åt enligt rekommendationerna för livsmedelsintag</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> med undantag för rekommendationerna om fisk samt sötsaker. De flesta barnen nådde även upp till rekommendationerna om fysisk aktivitet. De flesta mödrar ammade inte sina barn efter rekommendationerna. Det utlästes en signifikant skillnad mellan hur länge barnen ammats totalt och hur ofta de åt sötsaker som visade att barn som ammats under sex månader hade ett högre intag än de som ammats längre. (p=0</t>
+  </si>
+  <si>
+    <t>033) Barnen åt enligt rekommendationerna för de flesta livsmedel</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> utom fisk</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> som barnen åt mer sällan än vad som rekommenderas</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> samt sötsaker</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> som intogs oftare. Den information som framkommit i denna studie kan förtydliga vikten av att börja ett hälsofrämjande arbete i tidig ålder för att grundlägga goda vanor som sedan följer med barnen genom livet."</t>
+  </si>
+  <si>
+    <t>Tidigare studier visar att amningens längd kan påverka barns hälsa senare i livet. Även den sociala kontexten i familjen har kopplats till både hälsa och utveckling av matvanor. Salut är en folkhälsosatsning i Västerbotten med ambitionen att stärka befolkningens hälsa fram till år 2030. Målet med denna studie var att kartlägga matvanor, Body Mass Index (BMI) och fysisk aktivitet hos treåringar och analysera dessa i förhållande till amningsduration samt familjekonstellation.</t>
+  </si>
+  <si>
+    <t>Datainsamlingen skedde i samverkan med Salut</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> som tog fram en enkät och distribuerade den via barnavårdscentraler till föräldrar i samband med treårskontrollen. Enkäten omfattade frågor om barnens fysiska och psykiska hälsa samt levnadsvanor. Totalt inkluderades 210 enkäter i analysen</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> där 16 utvalda frågor bearbetades. Statistiska analyser genomfördes i IBM SPSS Statistics 21.0 och signifikansnivån sattes till p&lt;0</t>
+  </si>
+  <si>
+    <t>05. Resultaten visade att majoriteten av barnen följde rekommendationer för de flesta livsmedelsgrupper</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> men avvek gällande fisk och sötsaker. De flesta barn uppnådde även rekommenderad nivå av fysisk aktivitet. Däremot ammade flertalet mödrar inte i enlighet med rekommendationerna. En signifikant skillnad påvisades mellan total amningslängd och frekvens av sötsaksintag</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> där barn som ammats i sex månader hade ett högre intag än barn som ammats längre (p=0</t>
+  </si>
+  <si>
+    <t>033). Sammantaget följde barnen rekommendationerna för de flesta livsmedel</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> men åt fisk mer sällan och sötsaker oftare än rekommenderat. Studien kan bidra till att tydliggöra värdet av tidiga hälsofrämjande insatser för att etablera goda vanor som kan bestå genom livet."</t>
+  </si>
+  <si>
+    <t>Densitetsbestämningar och permeabilitetsprovning enligt EN 927-5 genomfördes för att undersöka om granvirkets fysiska karaktär i samspel med olika färgsystem påverkar materialets permeabilitet. I studien ingick jämförelser mellan frodvuxen och senvuxen ved, splintved och kärnved samt varierande densitet. De ytbehandlingar som utvärderades var alkyd-, akrylat- och linoljefärg, vilka ställdes mot en omålad kontroll. Resultaten visar ingen tydlig koppling mellan densitet och permeabilitet, vare sig för obehandlat eller målat virke. Däremot framstår vedens typ—splint kontra kärna samt frod- kontra senvuxenhet—som avgörande för vattenupptaget. Bestruken senvuxen kärnved uppvisade högst vattenabsorption för samtliga färgsystem. Vilken vedtyp som gav lägst absorption skiftade mellan systemen. Linolja gav överlag lägst permeabilitet, särskilt på frodvuxen kärnved, och denna kombination hade genomgående det minsta vattenupptaget under hela försöksperioden.</t>
+  </si>
+  <si>
+    <t>Den äldre typen av båsladugård har i stor utsträckning ersatts av lösdriftstallar där korna kan röra sig fritt och har ständig tillgång till foderbord och liggytor. Mjölkningen sker vanligtvis i mjölkgrop, karusell eller med hjälp av mjölkrobot. För att skapa god termisk komfort i dessa stall används antingen naturlig eller mekanisk ventilation. I detta arbete studeras flera lösningar för naturlig ventilation i fem utvalda kostall för att bedöma hur systemen fungerar i praktiken. Undersökningen genomförs med mätningar av temperatur och luftfuktighet samt med rökpatroner för att visualisera luftens rörelser i byggnaden. Resultaten jämförs och analyseras för att identifiera om något av ventilationssystemen presterar tydligt bättre eller sämre än de övriga. Avslutningsvis diskuteras även möjliga angreppssätt för att vidareutveckla studien i framtida arbete.</t>
+  </si>
+  <si>
+    <t>Denna uppsats undersöker barns sexualitet i förskolans kontext. Syftet är att synliggöra och problematisera hur förskolebarns sexualitet förstås samt att analysera vilka möjligheter och begränsningar förskollärare har att arbeta med området utifrån utvalda styr- och policydokument, och hur detta i förlängningen kan påverka barns utveckling. För att besvara studiens frågor används en kvalitativ innehållsanalys. Som jämförelsegrund används både förskolans och grundskolans läroplaner för att urskilja hur frågor om sex och samlevnad formuleras inom olika delar av utbildningssystemet. Därtill inkluderas Malmö högskolas utbildningsplan för att belysa hur förskollärarutbildningen behandlar barns sexualitet, samt ett dokument som redogör för en kommittés uppdrag och förslag till måldokument för pedagogiska verksamheter. De teoretiska utgångspunkterna tar avstamp i Foucaults syn på sexualitet, kompletterat med Donzelots resonemang om normer och moral samt begreppet normalisering. Resultaten indikerar att trots kravet på att förskolans praktik ska vila på forskning och beprövad erfarenhet erbjuds förskollärare i begränsad utsträckning utbildning i sex- och samlevnadsfrågor. I uppsatsen diskuteras möjliga förklaringar till att området tenderar att göras osynligt i förskolans sammanhang. Samtidigt argumenteras för att sex- och samlevnad kan integreras i förskolans arbete utan att läroplanen behöver omformuleras, och att detta kan stärka barns utveckling. Vinsterna beskrivs som ökad sexuell hälsa, en mer positiv självbild, kunskap om kroppslig integritet och sociala koder samt en bättre förståelse för egna känslor. Pedagoger ges också förutsättningar att motverka begränsande könsnormer och bidra till en mer tillåtande förskolemiljö. Om förskolan aktivt arbetar med sex- och samlevnad minskar risken att barn lämnas ensamma att hantera och tolka sina sexuella upplevelser och känslor.</t>
+  </si>
+  <si>
+    <t>Denna studie syftar till att fördjupa förståelsen för vad som kännetecknar mer utvecklade manliga skribenter i mellanstadiet. Med hjälp av en enkät om pojkars inställning till skrivande samt observationer av deras skrivande före och under ett längre skrivarbete undersöktes vilka faktorer som skiljer dessa elever från övriga i klassen. Resultaten visar att de mer avancerade skrivarna oftare har en bakgrund i hem med hög utbildningsnivå och att deras positiva syn på skrivande i stor utsträckning stöds och bekräftas av familjen. Vidare framkom att dessa pojkar i högre grad än sina kamrater lägger ner ansträngning både för sin egen skull och för att motsvara lärarens och vårdnadshavarnas förväntningar. Studien drar slutsatsen att hemmets värderingar i kombination med tydliga och höga lärarförväntningar hänger samman med en starkare motivation att anstränga sig för att utvecklas, vilket framstår som en avgörande faktor för att bli en mer avancerad skribent.</t>
+  </si>
+  <si>
+    <t>Utifrån ett symboliskt interaktionistiskt synsätt förstås människan som en social aktör i ett samhälle som ständigt blir till. Genom vardaglig interaktion formas individen samtidigt som individen bidrar till att skapa samhället, och just denna ömsesidighet utgör den röda tråden i antologin. I fyra bidrag undersöks olika livsomställningar och hur de påverkar självbild och livsvillkor. Agnesa Abrashi skriver i ”Ett nytt skede i livet – en studie om identitet och moderskap” om hur mödrar upplever sitt identitetsskapande i relation till moderskapet. Annika Sternlund behandlar adopterades erfarenheter av identitet och tillvaro i ”Rötterna är där hjärtat rotar sig”. I ”Som barn var man ju förväntansfull – en studie om individer som immigrerat vid unga år” skildrar Amanda Sundberg fem personers brytpunkter i livet i samband med migration i ung ålder. Helenas Valentinsons text ”Man känner ju i benen och det att man inte är 17 år längre” fokuserar på de förändringar som uppstår när man går i pension. Antologin förenas även av ett genomgående intresse för hur identitet formas i spänningsfältet mellan tillhörighet och utanförskap. Sammantaget visar studien att livsfaser och skiftande villkor påverkar identitetsskapandet, vilket gör identiteten att betrakta som föränderlig över tid.</t>
+  </si>
+  <si>
+    <t>Studien undersöker ur yrkesverksammas perspektiv hur urvalsprocessen och mottagandet av kvotflyktingar går till, samt hur samarbetet mellan de aktörer som arbetar med frågan fungerar. Arbetet är indelat i fyra delar: den första behandlar processen och samverkansformerna mellan berörda aktörer. Den andra delen fokuserar på samverkansutmaningar, följder av dessa och hur olika aktörer tolkar och värderar arbetet. I den tredje delen analyseras likheter och skillnader mellan kvotflyktingar och andra grupper av flyktingar. Den avslutande delen belyser hur lagstiftning och urvalskriterier påverkar förutsättningarna och besluten i processen.</t>
+  </si>
+  <si>
+    <t>Efter att Moderaterna tillsammans med övriga Allianspartier vann riksdagsvalet 2006 stod det klart att Sverige skulle få en omorienterad arbetsmarknadspolitik. Reformeringar av bland annat arbetslöshetsförsäkringen genomfördes i syfte att stärka drivkrafterna för arbetssökande att ta ett erbjudet arbete. Ersättningen skulle i mindre grad fungera som en långsiktig försörjning och i högre grad bidra till att arbete framstår som det mest lönsamma alternativet. Men vilka följder får dessa förändringar för de personer som omfattas av dem? Och på vilket sätt formas föreställningar om dessa personer i studiens empiriska underlag? Studiens mål är därför att granska hur Moderaterna beskriver och kategoriserar grupper utanför arbetsmarknaden, exempelvis arbetslösa och personer med sjuk- eller förtidspension. Vidare analyseras vilka åtgärder partiet föreslår för att hantera problemet samt vilka effekter dessa lösningar kan få för individers villkor när de står utanför arbetslivet.</t>
+  </si>
+  <si>
+    <t>Inom forskningen om public relations och strategisk kommunikation beskrivs ett paradigmskifte. Kommunikation förstås i allt mindre grad som ett budskap som överförs från en aktiv avsändare till en passiv mottagare, och i allt högre grad som något som formas i samspel mellan aktörer. Perspektivet förskjuts därmed från publiken som en påverkbar målgrupp till publiken som medskapare och deltagare i dialog. Men har denna förskjutning också fått genomslag i praktiken? Hur definieras och värderas kommunikation i svenska offentliga organisationer i dag? Vilka likheter och skillnader i synsätt kan urskiljas, och vilka förklaringar kan ligga bakom dem? Studien bygger på elva svenska offentliga organisationers kommunikationspolicys. Den teoretiska ramen utgörs av två svenska forskningsantologier om public relations respektive strategisk kommunikation samt ett urval kritiska och problematiserande artiklar. Efter en genomgång av litteraturen har centrala samtida forskningspositioner sammanställts. Med utgångspunkt i dessa konstruerades en idéanalytisk typologi baserad på två idealtyper. Resultaten visar tydliga mönster: nästan alla organisationer kunde sorteras in i någon av idealtyperna och synsätten hängde nära samman med hur organisationerna uttryckte sitt kommunikationsuppdrag. Samtliga forskningsperspektiv utom ett återfanns i materialet. Skillnaderna kunde i stor utsträckning relateras till organisationernas uppdrag och struktur. Organisationer som uttrycker mer dialogiska synsätt kännetecknas ofta av ett uttalat behov av att kommunicera effektivt med sin omvärld, medan övriga främst betonar kommunikation som informationsspridning.</t>
+  </si>
+  <si>
+    <t>Syftet med denna studie var att fördjupa förståelsen för och belysa hur sex förskolepedagoger upplever arbetet med att inkludera asylsökande barn i den ordinarie förskoleverksamheten, samt att beskriva hur pedagogerna menar att arbetet kring dessa barn planeras och genomförs. För att besvara studiens frågeställningar användes kvalitativa intervjuer. Intervjuerna utformades utifrån två övergripande forskningsfrågor som vägledde frågekonstruktionen: vilka villkor och möjligheter pedagogerna beskriver i arbetet med asylbarn, och hur förskolan organiseras för att möta asylbarn i den ordinarie verksamheten. Som analytiska perspektiv användes sociokulturell teori och interkulturell teori. Resultaten visar att integreringen innebär utmaningar kopplade till samarbete med barn och vårdnadshavare när gemensamt språk saknas och när pedagogerna har begränsad kunskap om familjernas bakgrund. Vidare behöver pedagogerna hantera barngrupper som ofta förändras och där närvaro och gruppstorlek kan variera från dag till dag. Studien visar även att ambitionen att asylbarn ska ges möjlighet att delta dagligen samtidigt kan innebära att vistelsetiden blir så kort att det försvårar ett mer strukturerat och långsiktigt arbete med barnens språkutveckling och deras kulturella erfarenheter.</t>
+  </si>
+  <si>
+    <t>Kvinnor och män har genom historien tillskrivits skilda kroppsliga och mentala egenskaper, och de samhälleliga normerna har i stor utsträckning utgått från mannen. Kvinnans roll har traditionellt varit knuten till hemmet som hustru, mor och ansvarig för hushållet. När samhället förändrades omformades också den könsuppdelade arbetsdelningen och fler kvinnor började arbeta utanför hemmet. Ämnet hem- och konsumentkunskap har samtidigt utvecklats från ett tidigare flickdominerat skolämne till ett obligatoriskt ämne för alla elever, där skolans uppdrag omfattar att främja jämställdhet mellan könen. Syftet med denna studie är att belysa hur verksamma lärare i hem- och konsumentkunskap uppfattar genus och jämställdhet i relation till ämnet, vilka faktorer som påverkar deras arbete med jämställdhet i undervisningen samt hur detta tar sig uttryck i praktiken. Sju legitimerade lärare i norra Sverige intervjuades individuellt. Deltagarna hade varierande ålder och yrkeserfarenhet. Intervjuerna ljudinspelades, skrevs ut och analyserades genom kvalitativ innehållsanalys. Lärarna beskrev att stereotypa föreställningar om kön är under förändring både i skolan och i hemmet, men att traditionella könsroller fortfarande återskapas. Hem- och konsumentkunskap framhölls som ett ämne där mycket av lärandet sker i praktiska moment, vilket gör att elevers roller och beteenden blir synliga och kan användas som utgångspunkt för samtal och reflektion kring jämställdhet. Samtidigt betonade lärarna att jämställdhetsarbete ställer höga krav på läraren, där den egna medvetenheten och den professionella rollen blir centrala, exempelvis i hur flickors och pojkars prestationer bedöms. Studiens slutsats är att lärare i hem- och konsumentkunskap upplever att könsstereotyper har försvagats, men att traditionella mönster fortsatt reproduceras i skolmiljön. Yngre generationer tycks i ökande grad bryta mot könsroller när jämställdhet blir mer självklar i samhället, men fortsatt utvecklingsarbete behövs eftersom skillnader mellan könen fortfarande syns, bland annat i betygsresultat.</t>
+  </si>
+  <si>
+    <t>Denna studies syfte är att utforska hur elever i årskurs nio ser på begreppet hälsa. Eftersom undervisningen i ämnet Idrott och hälsa kan utformas på skilda sätt vill studien också ge en tydligare bild av hur eleverna upplever att hälsofrågor behandlas i undervisningen. Med hjälp av intervjuer undersöks elevernas tankar och erfarenheter kring hälsa, samt vilka områden de önskar fördjupa sina kunskaper inom. Vidare efterfrågas deras uppfattningar om vad som är betydelsefullt för att kunna påverka den egna hälsan på längre sikt.</t>
+  </si>
+  <si>
+    <t>I den här studien har jag undersökt hur handledning tar sig uttryck på arbetsplatser. Handledning är i dag ett svårfångat begrepp som samtidigt blir allt vanligare i organisatoriska sammanhang. Arbetets mål är att belysa handledning och olika former av handledningsprocesser samt pröva hur dessa kan användas i arbetslivet, särskilt kopplat till medarbetarsamtalet. Jag avgränsar mig till den del av medarbetarsamtalet som handlar om medarbetarens utveckling. Min teoretiska utgångspunkt är att handledande inslag kan förekomma i medarbetarsamtal, men att hela samtalet inte självklart kan likställas med handledning. För att undersöka detta genomförde jag intervjuer med åtta personer på två arbetsplatser, där hälften var chefer och hälften medarbetare, med fokus på deras erfarenheter av medarbetarsamtal. Resultaten visar att ett handledande förhållningssätt tydligt kan identifieras i medarbetarsamtalen på båda arbetsplatserna och att metoder och perspektiv från handledningsfältet kan bidra till att vidareutveckla samtalets kvalitet och funktion. Om medarbetarsamtalet inte ses som handledning i sin helhet, men som en arena där handledning kan initieras, kan det förstås som en startpunkt för den mer kontinuerliga handledning som sker i vardagsarbetet. Samtalet blir då ett gemensamt tillfälle att klargöra förväntningar, enas om utvecklingsbehov och skapa en övergripande bild av arbetssituationen. Utifrån detta kan chef och medarbetare arbeta vidare med överenskomna frågor i det dagliga arbetet fram till nästa medarbetarsamtal.</t>
+  </si>
+  <si>
+    <t>Denna studie undersöker hur anställningsbarhet hänger samman med personlighet och arbetssökningsbeteende. Målgruppen är tidigare studenter från Arbetsvetenskapliga programmet vid Högskolan i Halmstad. Studien söker svar på om vissa personlighetsdrag ger fördelar i jobbsökandet, vilka kompetens- och personkrav som dominerar inom yrkesområdet samt om det finns samband mellan personlighet, anställningsbarhet och agerande i sökprocessen. För att kartlägga efterfrågade krav analyserades platsannonser och sammanställdes utifrån återkommande kriterier. Därutöver genomfördes en enkät med alumner och kompletterande intervjuer för att fördjupa förståelsen av deras erfarenheter. Resultaten indikerar att egenskaper kopplade till samvetsgrannhet och extroversion framträder som särskilt efterfrågade i annonserna. En majoritet av dem som arbetar inom området uppger att de fått sin tjänst via sociala kontakter. Intervjuerna visar också att deltagarna upplever att arbetsgivare fäster stor vikt vid personlighet vid rekrytering. Vidare framkommer att arbetslösa respondenter tenderar att vara mer proaktiva i sitt sökbeteende än övriga. Studien pekar även på tydliga samband mellan kön, familjesituation och geografisk rörlighet. Sammantaget tyder resultaten på att ett strategiskt arbetssätt och ett omfattande nätverk är centrala faktorer på vägen till relevant arbete, medan individuella skillnader inom gruppen i övrigt tycks spela mindre roll.</t>
+  </si>
+  <si>
+    <t>Denna uppsats har haft som mål att synliggöra behandlares syn på hur syskon och partners upplever att stå nära en person med ätstörning, samt vilken roll deras delaktighet kan ha i den drabbades behandlingsprocess. Studien har genomförts med en kvalitativ ansats där sex behandlare från olika svenska ätstörningsverksamheter intervjuades genom semistrukturerade intervjuer. Resultatet och slutsatserna pekar på att syskon, partners och andra närstående utgör en viktig resurs i patientens återhämtning. Därför behöver de inkluderas i behandlingen och erbjudas tydlig information om diagnos, förlopp och behandlingsupplägg. Syskon bör inte hamna i en överdriven ansvarsposition, medan partner ofta behöver ta ett visst praktiskt ansvar i vardagen. Ätstörningen påverkar i hög grad både partners och syskon, liksom närstående generellt. Närstående bör få konkreta verktyg för hur de kan stötta på ett hjälpsamt sätt. Behandlare bör möta närstående med respekt, förståelse och utan skuldbeläggning. En nära och fungerande relation mellan patienten och de involverade närstående framstår som betydelsefull för motivation och tillfrisknande. Samtidigt framkommer att forskningsläget är begränsat, vilket motiverar fortsatt forskning för att fördjupa och stärka dessa resultat.</t>
+  </si>
+  <si>
+    <t>Turismen i Kalmar har vuxit under senare år, men staden hamnar ofta i bakgrunden jämfört med Öland och Glasriket. Hur kan man få fler att se Kalmar som det självklara huvudresmålet och vad får dem att stanna längre? I den här uppsatsen undersöker vi hur ett starkt platsvarumärke byggs upp och vilka förutsättningar som krävs för att utvecklas till en attraktiv och konkurrenskraftig destination. Vi studerar även hur platsmarknadsföring kan användas för att kommunicera platsvarumärket och nå ut till relevanta målgrupper.</t>
+  </si>
+  <si>
+    <t>Under senare år har hållbarhetsfrågor blivit allt mer framträdande i samhället, och särskilt diskussionen om klimatpåverkan har fått stor uppmärksamhet. I takt med detta har företag mött ökade förväntningar från omvärlden att ta ett tydligare miljöansvar. Ett sätt att systematisera arbetet är att införa ett miljöledningssystem, och i samband med implementeringen väljer många företag att certifiera sig – något som också i växande grad efterfrågas av kunder. Trots detta är det fortfarande främst större organisationer som miljörapporterar och använder gröna nyckeltal för att synliggöra sin påverkan för intressenter. Bland mindre företag är sådan rapportering betydligt mindre utbredd. Utifrån denna bakgrund formulerades vår frågeställning: Vilka faktorer får små företag att införa miljöledningssystem och använda gröna nyckeltal, och hur organiserar de sitt praktiska miljöarbete?</t>
+  </si>
+  <si>
+    <t>Empirin samlades in genom en kombination av kvantitativ och kvalitativ metod. Den kvantitativa delen gav en övergripande bild och fungerade även som grund för urvalet till de kvalitativa intervjuerna. Analysen</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> förankrad i den teoretiska referensramen</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> visar att externa krav och intressentpåverkan ofta är centrala när miljöarbete initieras och när miljöledningssystem införs</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> medan interna nyttor senare blir de mest värderade. Resultaten indikerar att mindre företag upplever ett tryck att miljöcertifiera sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> men att certifiering i praktiken tycks spela en mindre roll vid upphandlingar än vad som ofta antas. Implementeringen av ett miljöledningssystem gör däremot miljöarbetet tydligare</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> mer konkret och mer strukturerat. När det gäller gröna nyckeltal dominerar energianvändning i olika former</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> men det framkommer svårigheter i att koppla dessa mått till verksamheten på ett enkelt</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> jämförbart och rättvisande sätt."</t>
+  </si>
+  <si>
+    <t>Barn som inte fyllt 15 år kan enligt 1 kap. 6 § BrB inte hållas straffrättsligt ansvariga för gärningar de begår. Trots detta kan ett skadeståndsrättsligt krav aktualiseras i en civilprocess i stort sett utan hänsyn till skadevållarens ålder. Utgångspunkten är därmed att även barn kan bli skadeståndsskyldiga på liknande sätt som vuxna, förutsatt att de anses ha orsakat skadan. De mest framträdande skillnaderna vid bedömningen av barns ansvar är dels att skadeståndet kan jämkas genom en särskild skälighetsprövning, dels att culpabedömningen anpassas och typiskt sett ställer lägre krav på barnets subjektiva förutsättningar. I uppsatsen analyseras även vårdnadshavares ansvar enligt 3 kap. 5 § skadeståndslagen, en bestämmelse som infördes 2010. Regeln innebär att föräldrar kan åläggas skadeståndsansvar för skador som barnet orsakar genom brott, och aktualiserar också kopplingen till tillsynsansvaret i 6 kap. 2 § föräldrabalken. Där anges att vårdnadshavaren ska ge barnet den tillsyn som krävs med hänsyn till ålder, mognad och övriga omständigheter för att förebygga skadevållande handlingar. En central skillnad mellan reglerna är att 3 kap. 5 § SkL tar sikte på brottsliga gärningar och inte kräver culpa, medan tillsynsansvaret kan bli relevant även utan att ett brott föreligger.</t>
+  </si>
+  <si>
+    <t>Inledning: Jordar förorenade med höga halter giftiga metaller till följd av antropogen verksamhet förekommer på flera platser på jorden och kan utgöra hälsorisk för både människor, djur och miljö. Därför finns orsak att se på miljövänliga metoder för sanering av förorenad mark. Då konventionella saneringsmetoder där jorden förflyttas från platsen ofta är mycket kostsamma och riskerar störa ekosystemen i hög grad är fytoremediering en metod med stor potential, vilken går ut på att rena mark eller vatten med växter. Studier har bland annat gjorts där annuell solros visat sig användbar för rening mark. Däremot verkar inga studier finns för perenn solros förmåga att ackumulera metaller från mark. Syfte: Syftet med studien är att undersöka perenn solros H. maximilianis upptag av metaller från jord hämtad från en åker i Mellansverige, samt att kvantifiera och kemiskt karakterisera metallerna i jorden. Frågeställningen studien ämnar besvara är om solrosen H. maximiliani lämpar sig för fytoremediering av metallförorenad mark. Metod: Perenn solros av sorten Helianthus maximiliani såddes i jord hämtad från en åker i Mellansverige och placerades i ett klimatreglerat växthus på Örebro universitet. Frön såddes samtidigt i såjord och vermiculit för senare omplantering till krukor med åkerjorden. Åkerjorden analyserades innan sådd på syralakbar halt metaller samt på växttillgänglig, reducerbar och oxiderbar halt. Plantorna skördades vid två tillfällen varpå metallinnehållet mättes för olika växtdelar. Jorden analyserades efter skörd. Metallanalysen gjordes i IPC-MS Agilent 7500 cx. Resultaten analyserades utifrån en signifikansnivå på 5 % och plantans ackumuleringseffektivitet beräknades och bedömdes utifrån BCF (bioconcentration factors). Resultat och slutsats: H. maximilianis tillväxt i åkerjorden var låg. Möjligtvis på grund av låg syrehalt och/eller lågt pH i jorden. H. maximiliani tog effektivt upp metaller som V, Cr, Co, Ni, Cu, Zn, Sr, Mo, Cd, Ba och Tl från den växttillgängliga fraktionen i marken till blad och stjälk. För att i realiteten kunna använda den perenna solrosen H maximiliani som fytoremedieringsgröda krävs högre tillväxt än vad som åstadkommits i studien. Åkerjorden från Kvinnersta innehöll halter av Cd, Cu, Zn och Ni högre än riktvärdena för acceptabel nivå innan slamgödsling bör ske, samt halter som översteg eller gränsade till riktvärdena för högsta acceptabla nivå för känslig markanvändning för metallerna As, Ba, Cd, Cu, och Zn. Halten uran var mellan cirka 5 och 50 gånger högre än den genomsnittliga uranhalten för jordar i Europa. De metaller av dem som förekom i hög halt i jorden (jämfört med Naturvårdsverkets gränsvärden för känslig markanvändning, samt gräns vid slamgödsling) som H. maximiliani inte tog upp effektivt var As, Pb och U.</t>
+  </si>
+  <si>
+    <t>**Inledning:** Mark som förorenats av höga halter toxiska metaller på grund av mänskliga aktiviteter förekommer globalt och kan innebära risker för människors och djurs hälsa samt för ekosystem. Detta motiverar utveckling och utvärdering av mer hållbara saneringsstrategier. Eftersom traditionella åtgärder, där jord schaktas bort och transporteras, ofta är mycket kostsamma och samtidigt kan orsaka omfattande ekologiska störningar, framstår fytoremediering som ett lovande alternativ. Metoden bygger på att växter används för att ta upp, binda eller stabilisera föroreningar i mark eller vatten. Tidigare forskning visar att ettårig solros kan bidra till metallrening, men kunskapsläget kring perenna solrosarters kapacitet att ackumulera metaller är begränsat.</t>
+  </si>
+  <si>
+    <t>**Syfte:** Studien syftar till att undersöka metallupptag hos den perenna solrosen *Helianthus maximilianis* i jord insamlad från en åker i Mellansverige</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> samt att kvantifiera och kemiskt fraktionera metallinnehållet i jorden. Den övergripande frågan är om *H. maximilianis* är en lämplig växt för fytoremediering av metallbelastad jord.</t>
+  </si>
+  <si>
+    <t>**Metod:** Frön av *Helianthus maximilianis* odlades i åkerjord under klimatkontrollerade växthusförhållanden vid Örebro universitet. Parallellt förgroddes frön i såjord och vermikulit för senare plantering i krukor med åkerjord. Före sådd analyserades jorden avseende syralakbar metallhalt samt fraktioner kopplade till växttillgänglig</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> reducerbar och oxiderbar del. Växtmaterial skördades vid två tidpunkter och metallhalter bestämdes i olika växtdelar; därefter analyserades jorden på nytt. Metallbestämningar utfördes med ICP‑MS (Agilent 7500 cx). Data utvärderades vid 5 % signifikansnivå och ackumulering bedömdes med biokoncentrationsfaktorer (BCF).</t>
+  </si>
+  <si>
+    <t>**Resultat och slutsats:** Tillväxten hos *H. maximilianis* i åkerjorden var svag</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> vilket kan ha påverkats av exempelvis syrebrist och/eller lågt pH. Trots detta uppvisade arten ett effektivt upptag från den växttillgängliga fraktionen av flera metaller (V</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Co</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ni</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Zn</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sr</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cd</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ba och Tl) till framför allt blad och stjälk. För praktisk användning som fytoremedieringsgröda krävs dock högre biomassatillväxt än den som uppnåddes här. Jorden från Kvinnersta hade Cd-</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cu-</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Zn- och Ni-halter över rekommenderade nivåer inför slamgödsling</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> och halter som överskred eller låg nära riktvärden för känslig markanvändning för As</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ba</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cu och Zn. Uranhalten var dessutom cirka 5–50 gånger högre än genomsnittet för europeiska jordar. Av de metaller som förekom i relativt höga halter var As</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Pb och U de som *H. maximilianis* inte ackumulerade effektivt."</t>
+  </si>
+  <si>
+    <t>Digital video har vuxit snabbt under de senaste åren. Tack vare moderna komprimeringstekniker kan i dag en hel långfilm lagras på en mobiltelefon eller en portabel mediaspelare. Men vad innebär videokompression i praktiken, och hur mycket kan en sekvens pressas utan att den upplevda nyttan går förlorad? I denna uppsats presenteras en översikt av de grundläggande principerna bakom videokompression. Kopplingen till upplevd användarnytta analyseras dessutom genom en experimentstudie. Där utvärderas tre videoklipp som kodats med tre olika kodekar och tre skilda bithastigheter, och resultaten jämförs mellan tre testgrupper. Studien visar att det är svårt att fastställa en tydlig gräns där kvaliteten blir oacceptabel för användaren. Samtidigt framgår att den högsta bithastigheten (256 kbit/s) ger hög användarnytta, medan den lägsta ger låg. Mellannivån 128 kbit/s bedöms som precis godtagbar av deltagarna.</t>
+  </si>
+  <si>
+    <t>Svenska språket bör vara tillgängligt för alla som lever och arbetar i Sverige. Därför behövs lättlästa versioner för personer som har svårt att ta till sig texter på svenska. Det här arbetet utgår från idén att automatisk omskrivning kan göra texter mer lättlästa och undersöker vidare hur ett sådant system kan byggas. Som grund används CogFLUX, ett verktyg som automatiskt skriver om text till lättare svenska genom syntaktiska förändringar. Omskrivningen styrs av regler som tagits fram i ett tidigare projekt. I detta arbete läggs nya omskrivningsregler till och dessutom utvecklas en ny modul som hanterar synonymval. Med hjälp av dessa tillägg analyseras om systemet kan producera texter som blir lättare enligt etablerade mått som LIX, OVIX och nominalkvot. Reglerna och synonymmodulen utvärderas på tre texter med en sammanlagd omfattning på cirka hundratusen ord. Resultaten visar att både LIX och nominalkvoten kan sänkas tydligt med omskrivningsregler och synonymhantering. Samtidigt indikerar studien att ytterligare utveckling krävs för att nå ett fullt välfungerande program för automatisk omskrivning till lätt svenska.</t>
+  </si>
+  <si>
+    <t>Tidigare studier har uppmärksammat flera typer av migrationsrelaterad språklig variation i svenskan, bland annat förortssvenska och förortsslang. Denna studie syftar till att kartlägga gymnasielärares sätt att beskriva dessa varieteter samt deras attityder till dem. Undersökningen genomförs med en enkät där lärarna får lyssna på utvalda språkprov och besvara frågor, följt av fokusgruppsdiskussioner. Examensarbetets empiri består av sju ifyllda enkäter och tre efterföljande fokusgruppssamtal som har spelats in och därefter grovtranskriberats. Resultaten visar en heterogen och delvis motsägelsefull bild. Talare av förortsslang bedömdes oftare som mindre ordningsamma, mindre sympatiska och mer “tuffa”, medan talare av förortssvenska i högre grad uppfattades som vänligare, mer ordentliga och mer intelligenta. Några lärare kunde känna igen förortssvenskan och särskilt notera dess prosodiska särdrag. Förortsslangen tolkades av vissa som ett bristande inlärarspråk, medan andra förstod den som en social markör kopplad till identitet och grupptillhörighet. Sammantaget pekar materialet på att den sociolingvistiska medvetenheten varierar tydligt mellan lärarna, från relativt utvecklad hos vissa till mer begränsad hos andra.</t>
+  </si>
+  <si>
+    <t>Denna uppsats undersöker eventkulturen inom det regionala resurscentrumet Film i Skåne. Studien tar sin teoretiska utgångspunkt i tidigare forskning om den svenska filmproduktionens regionalisering – en grundförutsättning för Film i Skånes verksamhet – samt i forskning om filmfestivalers betydelse för enskilda filmer och för deras ursprungsland eller region. Uppsatsens syfte är att klarlägga hur eventkulturen bidrar till Film i Skånes arbete och att identifiera vad, och vilka aktörer, som gynnas av denna eventinriktning. Tre typer av evenemang som Film i Skåne arrangerar eller samarrangerar beskrivs och analyseras för att synliggöra hur eventkulturen fungerar i praktiken. De evenemang som studeras är CineSkåne, M:Dox och Filmbar. Med stöd i de valda teoretiska perspektiven analyseras eventens roll och funktion i organisationens övergripande verksamhet. I avslutningen förs resonemang om att eventkulturen kan förstås som ett strategiskt verktyg för att stärka Film i Skånes position i det svenska filmlandskapet och samtidigt skapa förutsättningar för fortsatt tillväxt. Vidare argumenteras det för att eventkulturen stärker regionens filmklimat genom ett omfattande nätverk av arrangörer med geografisk räckvidd över stora delar av Skåne, samt att de mötesplatser och utvecklingsmöjligheter som evenemangen skapar är särskilt gynnsamma för verksamma filmarbetare.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -761,6 +1074,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -783,13 +1101,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1125,8 +1449,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B3FB63F-78D9-43E2-B34A-AB2BC4E7EF9C}">
-  <dimension ref="A1:H50"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I50"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
@@ -1135,10 +1459,11 @@
     <col min="5" max="5" width="105.36328125" customWidth="1"/>
     <col min="6" max="6" width="85.90625" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="50.1796875" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="67.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="67.1796875" customWidth="1"/>
+    <col min="9" max="9" width="17.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="2" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -1163,8 +1488,11 @@
       <c r="H1" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2">
         <v>2019</v>
       </c>
@@ -1190,7 +1518,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9">
       <c r="A3">
         <v>2014</v>
       </c>
@@ -1216,7 +1544,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -1242,7 +1570,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9">
       <c r="A5">
         <v>2010</v>
       </c>
@@ -1265,7 +1593,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -1282,7 +1610,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9">
       <c r="A7">
         <v>2014</v>
       </c>
@@ -1299,7 +1627,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9">
       <c r="A8">
         <v>2015</v>
       </c>
@@ -1316,7 +1644,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9">
       <c r="A9">
         <v>2015</v>
       </c>
@@ -1333,7 +1661,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9">
       <c r="A10">
         <v>2016</v>
       </c>
@@ -1350,7 +1678,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9">
       <c r="A11">
         <v>2015</v>
       </c>
@@ -1370,7 +1698,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9">
       <c r="A12">
         <v>2009</v>
       </c>
@@ -1390,7 +1718,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9">
       <c r="A13">
         <v>2017</v>
       </c>
@@ -1410,7 +1738,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9">
       <c r="A14">
         <v>2012</v>
       </c>
@@ -1430,7 +1758,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9">
       <c r="A15">
         <v>2013</v>
       </c>
@@ -1450,7 +1778,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9">
       <c r="A16">
         <v>2016</v>
       </c>
@@ -1470,7 +1798,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8">
       <c r="A17">
         <v>2015</v>
       </c>
@@ -1490,7 +1818,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8">
       <c r="A18">
         <v>2014</v>
       </c>
@@ -1510,7 +1838,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8">
       <c r="A19">
         <v>2010</v>
       </c>
@@ -1530,7 +1858,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8">
       <c r="A20">
         <v>2014</v>
       </c>
@@ -1550,7 +1878,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8">
       <c r="A21">
         <v>2007</v>
       </c>
@@ -1570,7 +1898,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8">
       <c r="A22">
         <v>2012</v>
       </c>
@@ -1590,7 +1918,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8">
       <c r="A23">
         <v>2008</v>
       </c>
@@ -1610,7 +1938,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8">
       <c r="A24">
         <v>2007</v>
       </c>
@@ -1630,7 +1958,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8">
       <c r="A25">
         <v>2016</v>
       </c>
@@ -1650,7 +1978,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8">
       <c r="A26">
         <v>2010</v>
       </c>
@@ -1670,7 +1998,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8">
       <c r="A27">
         <v>2017</v>
       </c>
@@ -1690,7 +2018,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8">
       <c r="A28">
         <v>2014</v>
       </c>
@@ -1710,7 +2038,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8">
       <c r="A29">
         <v>2015</v>
       </c>
@@ -1730,7 +2058,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8">
       <c r="A30">
         <v>2012</v>
       </c>
@@ -1750,7 +2078,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8">
       <c r="A31">
         <v>2014</v>
       </c>
@@ -1770,7 +2098,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8">
       <c r="A32">
         <v>2017</v>
       </c>
@@ -1790,7 +2118,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8">
       <c r="A33">
         <v>2011</v>
       </c>
@@ -1810,7 +2138,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8">
       <c r="A34">
         <v>2012</v>
       </c>
@@ -1830,7 +2158,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8">
       <c r="A35">
         <v>2007</v>
       </c>
@@ -1850,7 +2178,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8">
       <c r="A36">
         <v>2013</v>
       </c>
@@ -1870,7 +2198,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8">
       <c r="A37">
         <v>2013</v>
       </c>
@@ -1887,7 +2215,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8">
       <c r="A38">
         <v>2015</v>
       </c>
@@ -1904,7 +2232,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8">
       <c r="A39">
         <v>2013</v>
       </c>
@@ -1924,7 +2252,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8">
       <c r="A40">
         <v>2010</v>
       </c>
@@ -1944,7 +2272,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8">
       <c r="A41">
         <v>2010</v>
       </c>
@@ -1964,7 +2292,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8">
       <c r="A42">
         <v>2015</v>
       </c>
@@ -1984,7 +2312,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8">
       <c r="A43">
         <v>2012</v>
       </c>
@@ -2004,7 +2332,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8">
       <c r="A44">
         <v>2007</v>
       </c>
@@ -2024,7 +2352,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8">
       <c r="A45">
         <v>2016</v>
       </c>
@@ -2044,7 +2372,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8">
       <c r="A46">
         <v>2015</v>
       </c>
@@ -2064,7 +2392,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8">
       <c r="A47">
         <v>2007</v>
       </c>
@@ -2084,7 +2412,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8">
       <c r="A48">
         <v>2011</v>
       </c>
@@ -2104,7 +2432,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8">
       <c r="A49">
         <v>2016</v>
       </c>
@@ -2124,7 +2452,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8">
       <c r="A50">
         <v>2013</v>
       </c>
@@ -2162,4 +2490,1368 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId12"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4D2C4B4-81C6-4507-BF98-F02C67F2CA80}">
+  <dimension ref="A1:R65"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="144.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="255.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="168.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="5">
+        <v>2019</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="5">
+        <v>2014</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>156</v>
+      </c>
+      <c r="I3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="5">
+        <v>2017</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="5">
+        <v>2010</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="5">
+        <v>2014</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="5">
+        <v>2014</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="5">
+        <v>2016</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>97</v>
+      </c>
+      <c r="E10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="5">
+        <v>2009</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" t="s">
+        <v>82</v>
+      </c>
+      <c r="H12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="5">
+        <v>2017</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="5">
+        <v>2012</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" t="s">
+        <v>41</v>
+      </c>
+      <c r="I14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="5">
+        <v>2013</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="5">
+        <v>2016</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" t="s">
+        <v>53</v>
+      </c>
+      <c r="I16" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" t="s">
+        <v>51</v>
+      </c>
+      <c r="H17" t="s">
+        <v>41</v>
+      </c>
+      <c r="I17" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="5">
+        <v>2014</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" t="s">
+        <v>55</v>
+      </c>
+      <c r="H18" t="s">
+        <v>56</v>
+      </c>
+      <c r="I18" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" s="5">
+        <v>2010</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" t="s">
+        <v>59</v>
+      </c>
+      <c r="I19" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" s="5">
+        <v>2014</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" t="s">
+        <v>60</v>
+      </c>
+      <c r="H20" t="s">
+        <v>65</v>
+      </c>
+      <c r="I20" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" s="5">
+        <v>2007</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" t="s">
+        <v>64</v>
+      </c>
+      <c r="H21" t="s">
+        <v>41</v>
+      </c>
+      <c r="I21" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" s="5">
+        <v>2012</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" t="s">
+        <v>67</v>
+      </c>
+      <c r="H22" t="s">
+        <v>68</v>
+      </c>
+      <c r="I22" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" s="4"/>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="B24" t="s">
+        <v>182</v>
+      </c>
+      <c r="C24" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" s="5">
+        <v>2008</v>
+      </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" t="s">
+        <v>70</v>
+      </c>
+      <c r="H25" t="s">
+        <v>71</v>
+      </c>
+      <c r="I25" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" s="5">
+        <v>2007</v>
+      </c>
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" t="s">
+        <v>73</v>
+      </c>
+      <c r="D26" t="s">
+        <v>62</v>
+      </c>
+      <c r="E26" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26" t="s">
+        <v>74</v>
+      </c>
+      <c r="I26" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
+      <c r="A27" s="5">
+        <v>2016</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" t="s">
+        <v>75</v>
+      </c>
+      <c r="H27" t="s">
+        <v>77</v>
+      </c>
+      <c r="I27" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="A28" s="5">
+        <v>2010</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>79</v>
+      </c>
+      <c r="D28" t="s">
+        <v>81</v>
+      </c>
+      <c r="E28" t="s">
+        <v>78</v>
+      </c>
+      <c r="H28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I28" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29" s="5">
+        <v>2017</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" t="s">
+        <v>86</v>
+      </c>
+      <c r="I29" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30" s="5">
+        <v>2014</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" t="s">
+        <v>81</v>
+      </c>
+      <c r="E30" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="A31" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B31" t="s">
+        <v>191</v>
+      </c>
+      <c r="C31" t="s">
+        <v>192</v>
+      </c>
+      <c r="D31" t="s">
+        <v>193</v>
+      </c>
+      <c r="E31" t="s">
+        <v>194</v>
+      </c>
+      <c r="F31" t="s">
+        <v>195</v>
+      </c>
+      <c r="G31" t="s">
+        <v>196</v>
+      </c>
+      <c r="H31" t="s">
+        <v>197</v>
+      </c>
+      <c r="I31" t="s">
+        <v>198</v>
+      </c>
+      <c r="J31" t="s">
+        <v>199</v>
+      </c>
+      <c r="M31" t="s">
+        <v>87</v>
+      </c>
+      <c r="N31" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" s="4"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B33" t="s">
+        <v>202</v>
+      </c>
+      <c r="C33" t="s">
+        <v>203</v>
+      </c>
+      <c r="D33" t="s">
+        <v>204</v>
+      </c>
+      <c r="E33" t="s">
+        <v>205</v>
+      </c>
+      <c r="F33" t="s">
+        <v>206</v>
+      </c>
+      <c r="G33" t="s">
+        <v>207</v>
+      </c>
+      <c r="H33" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>90</v>
+      </c>
+      <c r="D34" t="s">
+        <v>81</v>
+      </c>
+      <c r="E34" t="s">
+        <v>91</v>
+      </c>
+      <c r="H34" t="s">
+        <v>92</v>
+      </c>
+      <c r="I34" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="5">
+        <v>2012</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" t="s">
+        <v>81</v>
+      </c>
+      <c r="E35" t="s">
+        <v>94</v>
+      </c>
+      <c r="H35" t="s">
+        <v>95</v>
+      </c>
+      <c r="I35" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="5">
+        <v>2014</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" t="s">
+        <v>98</v>
+      </c>
+      <c r="D36" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" t="s">
+        <v>99</v>
+      </c>
+      <c r="H36" t="s">
+        <v>100</v>
+      </c>
+      <c r="I36" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="5">
+        <v>2017</v>
+      </c>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>101</v>
+      </c>
+      <c r="D37" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" t="s">
+        <v>102</v>
+      </c>
+      <c r="H37" t="s">
+        <v>103</v>
+      </c>
+      <c r="I37" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="5">
+        <v>2011</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" t="s">
+        <v>106</v>
+      </c>
+      <c r="D38" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" t="s">
+        <v>104</v>
+      </c>
+      <c r="H38" t="s">
+        <v>105</v>
+      </c>
+      <c r="I38" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="5">
+        <v>2012</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" t="s">
+        <v>108</v>
+      </c>
+      <c r="D39" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" t="s">
+        <v>107</v>
+      </c>
+      <c r="H39" t="s">
+        <v>112</v>
+      </c>
+      <c r="I39" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="5">
+        <v>2007</v>
+      </c>
+      <c r="B40" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" t="s">
+        <v>110</v>
+      </c>
+      <c r="H40" t="s">
+        <v>111</v>
+      </c>
+      <c r="I40" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="5">
+        <v>2013</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
+        <v>113</v>
+      </c>
+      <c r="D41" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" t="s">
+        <v>114</v>
+      </c>
+      <c r="H41" t="s">
+        <v>115</v>
+      </c>
+      <c r="I41" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="5">
+        <v>2013</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" t="s">
+        <v>116</v>
+      </c>
+      <c r="D42" t="s">
+        <v>81</v>
+      </c>
+      <c r="E42" t="s">
+        <v>119</v>
+      </c>
+      <c r="I42" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B43" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" t="s">
+        <v>117</v>
+      </c>
+      <c r="D43" t="s">
+        <v>81</v>
+      </c>
+      <c r="E43" t="s">
+        <v>118</v>
+      </c>
+      <c r="I43" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="5">
+        <v>2013</v>
+      </c>
+      <c r="B44" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" t="s">
+        <v>120</v>
+      </c>
+      <c r="D44" t="s">
+        <v>81</v>
+      </c>
+      <c r="E44" t="s">
+        <v>121</v>
+      </c>
+      <c r="H44" t="s">
+        <v>122</v>
+      </c>
+      <c r="I44" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="5">
+        <v>2010</v>
+      </c>
+      <c r="B45" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" t="s">
+        <v>22</v>
+      </c>
+      <c r="D45" t="s">
+        <v>81</v>
+      </c>
+      <c r="E45" t="s">
+        <v>21</v>
+      </c>
+      <c r="H45" t="s">
+        <v>123</v>
+      </c>
+      <c r="I45" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="5">
+        <v>2010</v>
+      </c>
+      <c r="B46" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" t="s">
+        <v>124</v>
+      </c>
+      <c r="D46" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H46" t="s">
+        <v>126</v>
+      </c>
+      <c r="I46" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B47" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" t="s">
+        <v>127</v>
+      </c>
+      <c r="D47" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" t="s">
+        <v>128</v>
+      </c>
+      <c r="H47" t="s">
+        <v>129</v>
+      </c>
+      <c r="I47" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="5">
+        <v>2012</v>
+      </c>
+      <c r="B48" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" t="s">
+        <v>130</v>
+      </c>
+      <c r="D48" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" t="s">
+        <v>131</v>
+      </c>
+      <c r="H48" t="s">
+        <v>132</v>
+      </c>
+      <c r="I48" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18">
+      <c r="A49" s="5">
+        <v>2007</v>
+      </c>
+      <c r="B49" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" t="s">
+        <v>133</v>
+      </c>
+      <c r="D49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" t="s">
+        <v>134</v>
+      </c>
+      <c r="H49" t="s">
+        <v>135</v>
+      </c>
+      <c r="I49" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18">
+      <c r="A50" s="4"/>
+    </row>
+    <row r="51" spans="1:18">
+      <c r="A51" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18">
+      <c r="A52" s="4"/>
+    </row>
+    <row r="53" spans="1:18">
+      <c r="A53" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B53" t="s">
+        <v>226</v>
+      </c>
+      <c r="C53" t="s">
+        <v>227</v>
+      </c>
+      <c r="D53" t="s">
+        <v>228</v>
+      </c>
+      <c r="E53" t="s">
+        <v>229</v>
+      </c>
+      <c r="F53" t="s">
+        <v>230</v>
+      </c>
+      <c r="G53" t="s">
+        <v>231</v>
+      </c>
+      <c r="H53" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18">
+      <c r="A54" s="5">
+        <v>2016</v>
+      </c>
+      <c r="B54" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" t="s">
+        <v>138</v>
+      </c>
+      <c r="D54" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" t="s">
+        <v>136</v>
+      </c>
+      <c r="H54" t="s">
+        <v>137</v>
+      </c>
+      <c r="I54" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18">
+      <c r="A55" s="5">
+        <v>2015</v>
+      </c>
+      <c r="B55" t="s">
+        <v>9</v>
+      </c>
+      <c r="C55" t="s">
+        <v>140</v>
+      </c>
+      <c r="D55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E55" t="s">
+        <v>234</v>
+      </c>
+      <c r="H55" t="s">
+        <v>141</v>
+      </c>
+      <c r="I55" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18">
+      <c r="A56" s="4"/>
+    </row>
+    <row r="57" spans="1:18">
+      <c r="A57" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B57" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18">
+      <c r="A58" s="4"/>
+    </row>
+    <row r="59" spans="1:18">
+      <c r="A59" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="B59" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18">
+      <c r="A60" s="4"/>
+    </row>
+    <row r="61" spans="1:18">
+      <c r="A61" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="B61" t="s">
+        <v>241</v>
+      </c>
+      <c r="C61" t="s">
+        <v>242</v>
+      </c>
+      <c r="D61" t="s">
+        <v>243</v>
+      </c>
+      <c r="E61" t="s">
+        <v>244</v>
+      </c>
+      <c r="F61" t="s">
+        <v>245</v>
+      </c>
+      <c r="G61" t="s">
+        <v>246</v>
+      </c>
+      <c r="H61" t="s">
+        <v>247</v>
+      </c>
+      <c r="I61" t="s">
+        <v>248</v>
+      </c>
+      <c r="J61" t="s">
+        <v>249</v>
+      </c>
+      <c r="K61" t="s">
+        <v>250</v>
+      </c>
+      <c r="L61" t="s">
+        <v>251</v>
+      </c>
+      <c r="M61" t="s">
+        <v>252</v>
+      </c>
+      <c r="N61" t="s">
+        <v>253</v>
+      </c>
+      <c r="O61" t="s">
+        <v>254</v>
+      </c>
+      <c r="P61" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>255</v>
+      </c>
+      <c r="R61" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18">
+      <c r="A62" s="5">
+        <v>2007</v>
+      </c>
+      <c r="B62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" t="s">
+        <v>142</v>
+      </c>
+      <c r="D62" t="s">
+        <v>62</v>
+      </c>
+      <c r="E62" t="s">
+        <v>143</v>
+      </c>
+      <c r="H62" t="s">
+        <v>144</v>
+      </c>
+      <c r="I62" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18">
+      <c r="A63" s="5">
+        <v>2011</v>
+      </c>
+      <c r="B63" t="s">
+        <v>9</v>
+      </c>
+      <c r="C63" t="s">
+        <v>145</v>
+      </c>
+      <c r="D63" t="s">
+        <v>62</v>
+      </c>
+      <c r="E63" t="s">
+        <v>146</v>
+      </c>
+      <c r="H63" t="s">
+        <v>147</v>
+      </c>
+      <c r="I63" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18">
+      <c r="A64" s="5">
+        <v>2016</v>
+      </c>
+      <c r="B64" t="s">
+        <v>9</v>
+      </c>
+      <c r="C64" t="s">
+        <v>148</v>
+      </c>
+      <c r="D64" t="s">
+        <v>97</v>
+      </c>
+      <c r="E64" t="s">
+        <v>150</v>
+      </c>
+      <c r="H64" t="s">
+        <v>149</v>
+      </c>
+      <c r="I64" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9">
+      <c r="A65" s="5">
+        <v>2013</v>
+      </c>
+      <c r="B65" t="s">
+        <v>9</v>
+      </c>
+      <c r="C65" t="s">
+        <v>153</v>
+      </c>
+      <c r="D65" t="s">
+        <v>97</v>
+      </c>
+      <c r="E65" t="s">
+        <v>151</v>
+      </c>
+      <c r="H65" t="s">
+        <v>152</v>
+      </c>
+      <c r="I65" t="s">
+        <v>260</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>